<commit_message>
Joey Stella \$200 → Ben & Jack; raised \$1,385; ticker \$4,535
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -1463,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1878,23 +1878,43 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Joey Stella</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="16">
+      <c r="C23" s="16">
         <f>SUM(C4:C21)</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
         <is>
           <t>% of Goal</t>
         </is>
       </c>
-      <c r="C23" s="26">
+      <c r="C24" s="26">
         <f>C22/B2</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Eileen Linde \$100 → Jordana; raised \$729; ticker \$4,635
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -1883,11 +1883,6 @@
           <t>Mar 25</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Joey Stella</t>
-        </is>
-      </c>
       <c r="C22" s="20" t="n">
         <v>200</v>
       </c>
@@ -1934,7 +1929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2169,23 +2164,43 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Eileen Linde</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C13" s="16">
+      <c r="C14" s="16">
         <f>SUM(C4:C12)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>% of Goal</t>
         </is>
       </c>
-      <c r="C14" s="26">
+      <c r="C15" s="26">
         <f>C13/B2</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Excel: stripped to black/white/gray only
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,10 +34,10 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
-      <color rgb="00888888"/>
+      <color rgb="00999999"/>
       <sz val="9"/>
     </font>
     <font>
@@ -51,10 +51,6 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -65,7 +61,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEEE"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +75,7 @@
     </border>
     <border>
       <top style="medium">
-        <color rgb="00999999"/>
+        <color rgb="00AAAAAA"/>
       </top>
     </border>
     <border>
@@ -100,10 +96,10 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -478,10 +474,10 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>The Squeeze Project — Donations</t>
@@ -518,7 +514,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>% of Goal</t>
+          <t>% to Goal</t>
         </is>
       </c>
     </row>
@@ -676,7 +672,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Luke &amp; Aria Kerman — Camp IHC</t>
@@ -898,7 +894,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Tessa Forman — Camp Pontiac</t>
@@ -1300,7 +1296,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Ben &amp; Jack — Camp Wah-Nee</t>
@@ -1762,7 +1758,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Jordana Brody — Camp Westmont</t>
@@ -2024,7 +2020,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Parker Wellen — Camp Pontiac</t>

</xml_diff>

<commit_message>
Rebecca Brogadir \$100 → Ben & Jack; raised \$1,585; ticker \$4,835
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -1287,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1303,6 +1303,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1726,17 +1727,37 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Rebecca Brogadir</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n"/>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C24" s="8">
+      <c r="C25" s="8">
         <f>SUM(C4:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Stacey Selenfriend \$15 → Ben & Jack; raised \$1,620; ticker \$4,870
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -1509,7 +1509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2068,40 +2068,63 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Stacey Selenfriend</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Venmo</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C27" s="9">
+      <c r="C28" s="9">
         <f>SUM(C5:C25)</f>
         <v/>
       </c>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="10">
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="10">
         <f>SUM(E5:E25)</f>
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="15" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C28" s="16">
+      <c r="C29" s="16">
         <f>-E26</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="17" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C29" s="18">
+      <c r="C30" s="18">
         <f>C26+C27</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Kelly Hershkowitz \$50 Stripe → Ben & Jack; raised \$1,670; ticker \$5,020
</commit_message>
<xml_diff>
--- a/Squeeze_Project_Donations.xlsx
+++ b/Squeeze_Project_Donations.xlsx
@@ -756,7 +756,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1533,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1557,6 +1556,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2114,40 +2114,63 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="n"/>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Mar 25</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Kelly Hershkowitz</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>50</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Stripe</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C28" s="9">
+      <c r="C29" s="9">
         <f>SUM(C5:C25)</f>
         <v/>
       </c>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="10">
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="10">
         <f>SUM(E5:E25)</f>
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="15" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Est. Fees</t>
         </is>
       </c>
-      <c r="C29" s="16">
+      <c r="C30" s="16">
         <f>-E26</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="17" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>Net Received</t>
         </is>
       </c>
-      <c r="C30" s="18">
+      <c r="C31" s="18">
         <f>C26+C27</f>
         <v/>
       </c>

</xml_diff>